<commit_message>
Adding refactored data 20
</commit_message>
<xml_diff>
--- a/data/credit_exposure_inputs_raw.xlsx
+++ b/data/credit_exposure_inputs_raw.xlsx
@@ -521,7 +521,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Northbridge Manufacturing Ltd</t>
+          <t>Customer A</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -564,7 +564,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="L2" t="n">
@@ -601,7 +601,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Northbridge Manufacturing Ltd</t>
+          <t>Customer A</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -644,7 +644,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="L3" t="n">
@@ -681,7 +681,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Northbridge Manufacturing Ltd</t>
+          <t>Customer A</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -724,7 +724,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="L4" t="n">
@@ -761,7 +761,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Northbridge Manufacturing Ltd</t>
+          <t>Customer A</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -804,7 +804,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="L5" t="n">
@@ -841,7 +841,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Northbridge Manufacturing Ltd</t>
+          <t>Customer A</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -884,7 +884,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="L6" t="n">
@@ -921,7 +921,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Northbridge Manufacturing Ltd</t>
+          <t>Customer A</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -964,7 +964,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="L7" t="n">
@@ -1001,7 +1001,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Northbridge Manufacturing Ltd</t>
+          <t>Customer A</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1044,7 +1044,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="L8" t="n">
@@ -1081,7 +1081,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Northbridge Manufacturing Ltd</t>
+          <t>Customer A</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1124,7 +1124,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="L9" t="n">
@@ -1161,7 +1161,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Northbridge Manufacturing Ltd</t>
+          <t>Customer A</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1204,7 +1204,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="L10" t="n">
@@ -1241,7 +1241,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Calder Retail Group plc</t>
+          <t>Customer B</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1284,7 +1284,7 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="L11" t="n">
@@ -1321,7 +1321,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Calder Retail Group plc</t>
+          <t>Customer B</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1364,7 +1364,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="L12" t="n">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Calder Retail Group plc</t>
+          <t>Customer B</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1444,7 +1444,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="L13" t="n">
@@ -1481,7 +1481,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Calder Retail Group plc</t>
+          <t>Customer B</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1524,7 +1524,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="L14" t="n">
@@ -1561,7 +1561,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Calder Retail Group plc</t>
+          <t>Customer B</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1604,7 +1604,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="L15" t="n">
@@ -1641,7 +1641,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Meridian Logistics BV</t>
+          <t>Customer C</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1684,7 +1684,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="L16" t="n">
@@ -1721,7 +1721,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Meridian Logistics BV</t>
+          <t>Customer C</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1764,7 +1764,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="L17" t="n">
@@ -1801,7 +1801,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Tarvin Foods Ltd</t>
+          <t>Customer D</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1844,7 +1844,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="L18" t="n">
@@ -1881,7 +1881,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Tarvin Foods Ltd</t>
+          <t>Customer D</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1924,7 +1924,7 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="L19" t="n">
@@ -1961,7 +1961,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Tarvin Foods Ltd</t>
+          <t>Customer D</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2004,7 +2004,7 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="L20" t="n">
@@ -2041,7 +2041,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Tarvin Foods Ltd</t>
+          <t>Customer D</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2084,7 +2084,7 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="L21" t="n">
@@ -2121,7 +2121,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Tarvin Foods Ltd</t>
+          <t>Customer D</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2164,7 +2164,7 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="L22" t="n">
@@ -2201,7 +2201,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Tarvin Foods Ltd</t>
+          <t>Customer D</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2244,7 +2244,7 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="L23" t="n">
@@ -2281,7 +2281,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Tarvin Foods Ltd</t>
+          <t>Customer D</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2324,7 +2324,7 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="L24" t="n">
@@ -2361,7 +2361,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Tarvin Foods Ltd</t>
+          <t>Customer D</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -2404,7 +2404,7 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="L25" t="n">
@@ -2441,7 +2441,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Tarvin Foods Ltd</t>
+          <t>Customer D</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -2484,7 +2484,7 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="L26" t="n">
@@ -2521,7 +2521,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Tarvin Foods Ltd</t>
+          <t>Customer D</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -2564,7 +2564,7 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="L27" t="n">
@@ -2601,7 +2601,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Tarvin Foods Ltd</t>
+          <t>Customer D</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -2644,7 +2644,7 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="L28" t="n">
@@ -2681,7 +2681,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Halden Marine Ltd</t>
+          <t>Customer E</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -2724,7 +2724,7 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="L29" t="n">
@@ -2761,7 +2761,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Brackwell Utilities Ltd</t>
+          <t>Customer F</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2804,7 +2804,7 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="L30" t="n">
@@ -2841,7 +2841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Brackwell Utilities Ltd</t>
+          <t>Customer F</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -2884,7 +2884,7 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="L31" t="n">
@@ -2921,7 +2921,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Brackwell Utilities Ltd</t>
+          <t>Customer F</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -2964,7 +2964,7 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="L32" t="n">
@@ -3001,7 +3001,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Brackwell Utilities Ltd</t>
+          <t>Customer F</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -3044,7 +3044,7 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="L33" t="n">
@@ -3081,7 +3081,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Pelham Textiles Ltd</t>
+          <t>Customer G</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -3124,7 +3124,7 @@
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="L34" t="n">
@@ -3161,7 +3161,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Pelham Textiles Ltd</t>
+          <t>Customer G</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -3204,7 +3204,7 @@
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="L35" t="n">
@@ -3241,7 +3241,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Pelham Textiles Ltd</t>
+          <t>Customer G</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -3284,7 +3284,7 @@
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="L36" t="n">
@@ -3321,7 +3321,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Pelham Textiles Ltd</t>
+          <t>Customer G</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -3364,7 +3364,7 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="L37" t="n">
@@ -9221,7 +9221,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="I2" t="n">
@@ -9272,7 +9272,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="I3" t="n">
@@ -9323,7 +9323,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="I4" t="n">
@@ -9377,7 +9377,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -9431,7 +9431,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -9482,7 +9482,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -9533,7 +9533,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -9584,7 +9584,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -9635,7 +9635,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -9686,7 +9686,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -9737,7 +9737,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -9785,7 +9785,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -9836,7 +9836,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -9887,7 +9887,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -9935,7 +9935,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="I16" t="n">
@@ -9986,7 +9986,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="I17" t="n">
@@ -10037,7 +10037,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="I18" t="n">
@@ -10085,7 +10085,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="I19" t="n">
@@ -10136,7 +10136,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="I20" t="n">
@@ -10187,7 +10187,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="I21" t="n">
@@ -10238,7 +10238,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="I22" t="n">
@@ -10289,7 +10289,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="I23" t="n">

</xml_diff>